<commit_message>
FILE_CHECK starts FILE_LOAD for passed files; Facets 210 pulls; export to SDO feed tables (0.3.69)
- FILE_CHECK: when a file fails, check_passed still triggers the next DAGs if at
  least one file passed; file_check_result keeps the run failed.
- CMSUNIV: ODAG3 / FA4 source 210 pulled from CMSUNIV_CORE_DEV_V.CSF_* by Batch_ID,
  IDs by ROW_SEQUENCE; export rows write to EXPORT_FEED_$ENV_T.SDO_CMSUNIV_<table>_2022.
- Runbook, open items and test cases updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/airflow_resources/docs/TEST_CASES.xlsx
+++ b/airflow_resources/docs/TEST_CASES.xlsx
@@ -4289,7 +4289,7 @@
       <c r="I40" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -8302,7 +8302,7 @@
       <c r="I96" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -8372,7 +8372,7 @@
       <c r="I97" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -8380,7 +8380,7 @@
       </c>
       <c r="J97" s="13" t="inlineStr">
         <is>
-          <t>Exported the same day; EXPORT_LOADED; Q8 rows = core rows; Exp_Btch_ID = batch</t>
+          <t>Exported the same day; EXPORT_LOADED; Q8 rows = core rows; Btch_ID = batch</t>
         </is>
       </c>
       <c r="K97" s="15" t="inlineStr">
@@ -8413,7 +8413,7 @@
       </c>
       <c r="D98" s="13" t="inlineStr">
         <is>
-          <t>CMSUNIV procedure configured</t>
+          <t>A test table with Exp_Proc_Nm set (CMSUNIV itself has no procedure)</t>
         </is>
       </c>
       <c r="E98" s="13" t="inlineStr">
@@ -8433,7 +8433,7 @@
       <c r="H98" s="13" t="inlineStr">
         <is>
           <t>1. Check the precondition
-2. Prepare the input: CMSUNIV procedure configured
+2. Prepare the input: A test table with Exp_Proc_Nm set (CMSUNIV itself has no procedure)
 3. Run the job
 4. Run the verification SQL (replace &lt;batch&gt;, &lt;table&gt;)
 5. Compare with the expected result and record the outcome</t>
@@ -8442,7 +8442,7 @@
       <c r="I98" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -8450,7 +8450,7 @@
       </c>
       <c r="J98" s="13" t="inlineStr">
         <is>
-          <t>Log procedure CMSUNIV_EXPORT_DEV_T.SP_EXPORT_… with parameters; rows stamped Btch_ID / Exp_Btch_ID</t>
+          <t>Log procedure &lt;db&gt;.&lt;proc&gt; with parameters; rows stamped Btch_ID (and Exp_Btch_ID if present)</t>
         </is>
       </c>
       <c r="K98" s="15" t="inlineStr">
@@ -8512,7 +8512,7 @@
       <c r="I99" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -8582,7 +8582,7 @@
       <c r="I100" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -8652,7 +8652,7 @@
       <c r="I101" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -8722,7 +8722,7 @@
       <c r="I102" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -8792,7 +8792,7 @@
       <c r="I103" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -8862,7 +8862,7 @@
       <c r="I104" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -8932,7 +8932,7 @@
       <c r="I105" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -9002,7 +9002,7 @@
       <c r="I106" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -9072,7 +9072,7 @@
       <c r="I107" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -9142,7 +9142,7 @@
       <c r="I108" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -9183,7 +9183,7 @@
       </c>
       <c r="D109" s="13" t="inlineStr">
         <is>
-          <t>Remove Exp_Proc_Nm on a test table</t>
+          <t>CMSUNIV export rows as delivered (no procedure)</t>
         </is>
       </c>
       <c r="E109" s="13" t="inlineStr">
@@ -9208,7 +9208,7 @@
       <c r="H109" s="13" t="inlineStr">
         <is>
           <t>1. Check the precondition and run the setup SQL
-2. Prepare the input: Remove Exp_Proc_Nm on a test table
+2. Prepare the input: CMSUNIV export rows as delivered (no procedure)
 3. Run the job
 4. Run the verification SQL (replace &lt;batch&gt;, &lt;table&gt;)
 5. Compare with the expected result and record the outcome
@@ -9218,7 +9218,7 @@
       <c r="I109" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -9226,7 +9226,7 @@
       </c>
       <c r="J109" s="13" t="inlineStr">
         <is>
-          <t>Same-name core columns copied; Exp_Btch_ID filled; validate warns about export columns missing in core</t>
+          <t>Core columns copied into SDO_CMSUNIV_&lt;table&gt;_2022 by name, then value code, then order; Btch_ID = batch; validate lists the pairs and warns about feed columns no core column fills</t>
         </is>
       </c>
       <c r="K109" s="15" t="inlineStr">
@@ -9294,7 +9294,7 @@
       <c r="I110" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -9420,10 +9420,10 @@
       </c>
       <c r="F112" s="14" t="inlineStr">
         <is>
-          <t>CREATE TABLE CMSUNIV_EXPORT_DEV_T.Test_Steps (Step VARCHAR(10), Btch_ID VARCHAR(255), Run_Ty VARCHAR(15));
+          <t>CREATE TABLE EXPORT_FEED_DEV_T.Test_Steps (Step VARCHAR(10), Btch_ID VARCHAR(255), Run_Ty VARCHAR(15));
 UPDATE HSABC_DEV.ComplianceExportConfig SET
-  Exp_Pre_Sql_Txt = 'INSERT INTO CMSUNIV_EXPORT_DEV_T.Test_Steps VALUES (''pre'', {btch_id}, {run_ty})',
-  Exp_Post_Sql_Txt = 'INSERT INTO CMSUNIV_EXPORT_DEV_T.Test_Steps VALUES (''post'', {btch_id}, {run_ty})'
+  Exp_Pre_Sql_Txt = 'INSERT INTO EXPORT_FEED_DEV_T.Test_Steps VALUES (''pre'', {btch_id}, {run_ty})',
+  Exp_Post_Sql_Txt = 'INSERT INTO EXPORT_FEED_DEV_T.Test_Steps VALUES (''post'', {btch_id}, {run_ty})'
 WHERE Project_Cd = 'CMSUNIV' AND Table_Nm = '&lt;test table&gt;';</t>
         </is>
       </c>
@@ -9446,8 +9446,8 @@
       <c r="I112" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
-SELECT * FROM CMSUNIV_EXPORT_DEV_T.Test_Steps ORDER BY 1;</t>
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+SELECT * FROM EXPORT_FEED_DEV_T.Test_Steps ORDER BY 1;</t>
         </is>
       </c>
       <c r="J112" s="13" t="inlineStr">
@@ -9496,7 +9496,7 @@
       </c>
       <c r="F113" s="14" t="inlineStr">
         <is>
-          <t>UPDATE HSABC_DEV.ComplianceExportConfig SET Exp_Post_Sql_Txt = 'UPDATE CMSUNIV_EXPORT_DEV_T.No_Such_Table SET x = 1 WHERE y = {btch_id}'
+          <t>UPDATE HSABC_DEV.ComplianceExportConfig SET Exp_Post_Sql_Txt = 'UPDATE EXPORT_FEED_DEV_T.No_Such_Table SET x = 1 WHERE y = {btch_id}'
 WHERE Project_Cd = 'CMSUNIV' AND Table_Nm = '&lt;test table&gt;';</t>
         </is>
       </c>
@@ -9519,8 +9519,8 @@
       <c r="I113" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
-SELECT * FROM CMSUNIV_EXPORT_DEV_T.Test_Steps ORDER BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+SELECT * FROM EXPORT_FEED_DEV_T.Test_Steps ORDER BY 1;
 SELECT Event_ID, Event_Ty, Sevrty, Src_ID, Load_ID, Event_Txt, Notified_Ind
 FROM HSABC_DEV.CMS_ComplianceExceptionsAudit WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Event_ID;</t>
         </is>
@@ -9589,7 +9589,7 @@
       <c r="I114" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -9659,7 +9659,7 @@
       <c r="I115" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -9729,7 +9729,7 @@
       <c r="I116" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT COUNT(*) FROM EXPORT_FEED_DEV_V.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;';</t>
         </is>
       </c>
@@ -9797,7 +9797,7 @@
       <c r="I117" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -9868,7 +9868,7 @@
       <c r="I118" s="14" t="inlineStr">
         <is>
           <t>SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT c.Src_ID, d.Event_Dtts, d.Event_Ty, d.Load_ID, d.Event_Txt
 FROM HSABC_DEV.ComplianceRequestFileDetail d JOIN HSABC_DEV.ComplianceRequestControl c ON c.Req_ID = d.Req_ID
 WHERE c.Btch_ID = '&lt;batch&gt;' ORDER BY c.Src_ID, d.Detail_ID;</t>
@@ -13270,7 +13270,7 @@
 SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT rule_id, status, run_key FROM HSABC_DEV.gre_results WHERE run_key = '&lt;batch&gt;' ORDER BY 1;
 SELECT rule_id, run_type, batch_schedule, COUNT(*) FROM HSABC_DEV.gre_exceptions
 WHERE run_key = '&lt;batch&gt;' AND etl_is_curr_ind = 'Y' GROUP BY 1, 2, 3;</t>
@@ -13339,7 +13339,7 @@
 SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT rule_id, status, run_key FROM HSABC_DEV.gre_results WHERE run_key = '&lt;batch&gt;' ORDER BY 1;
 SELECT rule_id, run_type, batch_schedule, COUNT(*) FROM HSABC_DEV.gre_exceptions
 WHERE run_key = '&lt;batch&gt;' AND etl_is_curr_ind = 'Y' GROUP BY 1, 2, 3;</t>
@@ -13408,7 +13408,7 @@
 SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT rule_id, status, run_key FROM HSABC_DEV.gre_results WHERE run_key = '&lt;batch&gt;' ORDER BY 1;
 SELECT rule_id, run_type, batch_schedule, COUNT(*) FROM HSABC_DEV.gre_exceptions
 WHERE run_key = '&lt;batch&gt;' AND etl_is_curr_ind = 'Y' GROUP BY 1, 2, 3;</t>
@@ -13477,7 +13477,7 @@
 SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT rule_id, status, run_key FROM HSABC_DEV.gre_results WHERE run_key = '&lt;batch&gt;' ORDER BY 1;
 SELECT rule_id, run_type, batch_schedule, COUNT(*) FROM HSABC_DEV.gre_exceptions
 WHERE run_key = '&lt;batch&gt;' AND etl_is_curr_ind = 'Y' GROUP BY 1, 2, 3;</t>
@@ -13546,7 +13546,7 @@
 SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT rule_id, status, run_key FROM HSABC_DEV.gre_results WHERE run_key = '&lt;batch&gt;' ORDER BY 1;
 SELECT rule_id, run_type, batch_schedule, COUNT(*) FROM HSABC_DEV.gre_exceptions
 WHERE run_key = '&lt;batch&gt;' AND etl_is_curr_ind = 'Y' GROUP BY 1, 2, 3;</t>
@@ -13615,7 +13615,7 @@
 SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT rule_id, status, run_key FROM HSABC_DEV.gre_results WHERE run_key = '&lt;batch&gt;' ORDER BY 1;
 SELECT rule_id, run_type, batch_schedule, COUNT(*) FROM HSABC_DEV.gre_exceptions
 WHERE run_key = '&lt;batch&gt;' AND etl_is_curr_ind = 'Y' GROUP BY 1, 2, 3;</t>
@@ -13684,7 +13684,7 @@
 SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT rule_id, status, run_key FROM HSABC_DEV.gre_results WHERE run_key = '&lt;batch&gt;' ORDER BY 1;
 SELECT rule_id, run_type, batch_schedule, COUNT(*) FROM HSABC_DEV.gre_exceptions
 WHERE run_key = '&lt;batch&gt;' AND etl_is_curr_ind = 'Y' GROUP BY 1, 2, 3;</t>
@@ -13755,7 +13755,7 @@
 SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT rule_id, status, run_key FROM HSABC_DEV.gre_results WHERE run_key = '&lt;batch&gt;' ORDER BY 1;
 SELECT rule_id, run_type, batch_schedule, COUNT(*) FROM HSABC_DEV.gre_exceptions
 WHERE run_key = '&lt;batch&gt;' AND etl_is_curr_ind = 'Y' GROUP BY 1, 2, 3;</t>
@@ -13824,7 +13824,7 @@
 SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_
-FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;
+FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
 SELECT rule_id, status, run_key FROM HSABC_DEV.gre_results WHERE run_key = '&lt;batch&gt;' ORDER BY 1;
 SELECT rule_id, run_type, batch_schedule, COUNT(*) FROM HSABC_DEV.gre_exceptions
 WHERE run_key = '&lt;batch&gt;' AND etl_is_curr_ind = 'Y' GROUP BY 1, 2, 3;</t>
@@ -14391,7 +14391,7 @@
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>SELECT Src_Data_Key, COUNT(*) FROM CMSUNIV_EXPORT_DEV_T.&lt;table&gt;_EXPORT WHERE Exp_Btch_ID = '&lt;batch&gt;' GROUP BY 1;</t>
+          <t>SELECT Src_Data_Key, COUNT(*) FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;</t>
         </is>
       </c>
     </row>
@@ -14559,7 +14559,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Staging, core, export tables and export procedures created (examples/cmsuniv_export_dev.sql)</t>
+          <t>Staging and core tables created; feed tables EXPORT_FEED_DEV_T.SDO_CMSUNIV_* exist with Btch_ID and Src_Data_Key</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Audit columns renamed, tables reordered with audit columns last, LastUpdt_ID set to database user; one-time upgrade and schema check (0.3.71)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/airflow_resources/docs/TEST_CASES.xlsx
+++ b/airflow_resources/docs/TEST_CASES.xlsx
@@ -4218,7 +4218,7 @@
       </c>
       <c r="I39" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_ID, Req_Stat, Resolution_Ty, Batch_Close_Ind, Reuse_Btch_ID, Rpt_Start_Dt_Key, Rpt_End_Dt_Key
 FROM HSABC_DEV.ComplianceRequestControl WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Src_ID;</t>
@@ -5092,7 +5092,7 @@
       </c>
       <c r="I52" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -5165,7 +5165,7 @@
       </c>
       <c r="I53" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -5238,7 +5238,7 @@
       </c>
       <c r="I54" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -5311,7 +5311,7 @@
       </c>
       <c r="I55" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -5384,7 +5384,7 @@
       </c>
       <c r="I56" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -5457,7 +5457,7 @@
       </c>
       <c r="I57" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -5530,7 +5530,7 @@
       </c>
       <c r="I58" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -5603,7 +5603,7 @@
       </c>
       <c r="I59" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -5676,7 +5676,7 @@
       </c>
       <c r="I60" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -5749,7 +5749,7 @@
       </c>
       <c r="I61" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -5822,7 +5822,7 @@
       </c>
       <c r="I62" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -5895,7 +5895,7 @@
       </c>
       <c r="I63" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -5968,7 +5968,7 @@
       </c>
       <c r="I64" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -6045,7 +6045,7 @@
       </c>
       <c r="I65" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -6191,7 +6191,7 @@
       </c>
       <c r="I67" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -6264,7 +6264,7 @@
       </c>
       <c r="I68" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -6337,7 +6337,7 @@
       </c>
       <c r="I69" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -6410,7 +6410,7 @@
       </c>
       <c r="I70" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -6483,7 +6483,7 @@
       </c>
       <c r="I71" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -6556,7 +6556,7 @@
       </c>
       <c r="I72" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -6629,7 +6629,7 @@
       </c>
       <c r="I73" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Btch_ID, Src_Data_Key, Run_Ty, AuditDataID, COUNT(*) AS Rows_
 FROM CMSUNIV_FILELAND_DEV_T.&lt;staging table&gt; GROUP BY 1, 2, 3, 4 ORDER BY 1, 2;
@@ -6702,7 +6702,7 @@
       </c>
       <c r="I74" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_, MIN(StagingCreateDate), MAX(Load_Dtts)
 FROM CMSUNIV_CORE_DEV_T.&lt;core table&gt; WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -6772,7 +6772,7 @@
       </c>
       <c r="I75" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_, MIN(StagingCreateDate), MAX(Load_Dtts)
 FROM CMSUNIV_CORE_DEV_T.&lt;core table&gt; WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -6842,7 +6842,7 @@
       </c>
       <c r="I76" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_, MIN(StagingCreateDate), MAX(Load_Dtts)
 FROM CMSUNIV_CORE_DEV_T.&lt;core table&gt; WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -6912,7 +6912,7 @@
       </c>
       <c r="I77" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_, MIN(StagingCreateDate), MAX(Load_Dtts)
 FROM CMSUNIV_CORE_DEV_T.&lt;core table&gt; WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -6982,7 +6982,7 @@
       </c>
       <c r="I78" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_, MIN(StagingCreateDate), MAX(Load_Dtts)
 FROM CMSUNIV_CORE_DEV_T.&lt;core table&gt; WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -7052,7 +7052,7 @@
       </c>
       <c r="I79" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_, MIN(StagingCreateDate), MAX(Load_Dtts)
 FROM CMSUNIV_CORE_DEV_T.&lt;core table&gt; WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -7127,7 +7127,7 @@
       </c>
       <c r="I80" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_, MIN(StagingCreateDate), MAX(Load_Dtts)
 FROM CMSUNIV_CORE_DEV_T.&lt;core table&gt; WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -7197,7 +7197,7 @@
       </c>
       <c r="I81" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_, MIN(StagingCreateDate), MAX(Load_Dtts)
 FROM CMSUNIV_CORE_DEV_T.&lt;core table&gt; WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -7267,7 +7267,7 @@
       </c>
       <c r="I82" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_, MIN(StagingCreateDate), MAX(Load_Dtts)
 FROM CMSUNIV_CORE_DEV_T.&lt;core table&gt; WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -7337,7 +7337,7 @@
       </c>
       <c r="I83" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_, MIN(StagingCreateDate), MAX(Load_Dtts)
 FROM CMSUNIV_CORE_DEV_T.&lt;core table&gt; WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -7473,7 +7473,7 @@
       </c>
       <c r="I85" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_, MIN(StagingCreateDate), MAX(Load_Dtts)
 FROM CMSUNIV_CORE_DEV_T.&lt;core table&gt; WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -7543,7 +7543,7 @@
       </c>
       <c r="I86" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_, MIN(StagingCreateDate), MAX(Load_Dtts)
 FROM CMSUNIV_CORE_DEV_T.&lt;core table&gt; WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -7613,7 +7613,7 @@
       </c>
       <c r="I87" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_, MIN(StagingCreateDate), MAX(Load_Dtts)
 FROM CMSUNIV_CORE_DEV_T.&lt;core table&gt; WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -13267,7 +13267,7 @@
 FROM HSABC_DEV.ComplianceRequestControl
 WHERE Project_Cd = 'CMSUNIV' AND Req_Dt_Key = CURRENT_DATE
 ORDER BY Btch_ID, Src_ID;
-SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_
 FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -13336,7 +13336,7 @@
 FROM HSABC_DEV.ComplianceRequestControl
 WHERE Project_Cd = 'CMSUNIV' AND Req_Dt_Key = CURRENT_DATE
 ORDER BY Btch_ID, Src_ID;
-SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_
 FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -13405,7 +13405,7 @@
 FROM HSABC_DEV.ComplianceRequestControl
 WHERE Project_Cd = 'CMSUNIV' AND Req_Dt_Key = CURRENT_DATE
 ORDER BY Btch_ID, Src_ID;
-SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_
 FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -13474,7 +13474,7 @@
 FROM HSABC_DEV.ComplianceRequestControl
 WHERE Project_Cd = 'CMSUNIV' AND Req_Dt_Key = CURRENT_DATE
 ORDER BY Btch_ID, Src_ID;
-SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_
 FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -13543,7 +13543,7 @@
 FROM HSABC_DEV.ComplianceRequestControl
 WHERE Project_Cd = 'CMSUNIV' AND Req_Dt_Key = CURRENT_DATE
 ORDER BY Btch_ID, Src_ID;
-SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_
 FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -13612,7 +13612,7 @@
 FROM HSABC_DEV.ComplianceRequestControl
 WHERE Project_Cd = 'CMSUNIV' AND Req_Dt_Key = CURRENT_DATE
 ORDER BY Btch_ID, Src_ID;
-SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_
 FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -13681,7 +13681,7 @@
 FROM HSABC_DEV.ComplianceRequestControl
 WHERE Project_Cd = 'CMSUNIV' AND Req_Dt_Key = CURRENT_DATE
 ORDER BY Btch_ID, Src_ID;
-SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_
 FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -13752,7 +13752,7 @@
 FROM HSABC_DEV.ComplianceRequestControl
 WHERE Project_Cd = 'CMSUNIV' AND Req_Dt_Key = CURRENT_DATE
 ORDER BY Btch_ID, Src_ID;
-SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_
 FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -13821,7 +13821,7 @@
 FROM HSABC_DEV.ComplianceRequestControl
 WHERE Project_Cd = 'CMSUNIV' AND Req_Dt_Key = CURRENT_DATE
 ORDER BY Btch_ID, Src_ID;
-SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+SELECT Load_ID, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;
 SELECT Src_Data_Key, COUNT(*) AS Rows_
 FROM EXPORT_FEED_DEV_T.SDO_CMSUNIV_&lt;table&gt;_2022 WHERE Btch_ID = '&lt;batch&gt;' GROUP BY 1;
@@ -14321,7 +14321,7 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>SELECT Load_ID, File_Share, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, Updated_Dtts
+          <t>SELECT Load_ID, File_Share, File_Path, Load_Stat, Reject_Rsn_Cd, Rules_Stat, Stg_Rcd_Cnt, Error_Txt, LastUpdt_Dtts
 FROM HSABC_DEV.ComplianceFileLoad WHERE Btch_ID = '&lt;batch&gt;' ORDER BY Load_ID DESC;</t>
         </is>
       </c>

</xml_diff>